<commit_message>
Refactored ahm and medibank direct offers
</commit_message>
<xml_diff>
--- a/comp_offer.xlsx
+++ b/comp_offer.xlsx
@@ -1156,11 +1156,27 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>up to 12 weeks free</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>2 &amp; 6 month waiting periods on extras</t>
+        </is>
+      </c>
       <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
-      <c r="H10" s="12" t="n"/>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>30 jun 2026</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>General - offer for new joins Available for new members on new memberships who have not held ahm hospital and/or extras cover in the last 30 days from their cover start date (unless a dependant coming off a family cover or single parent family cover). Must join and commence an eligible hospital and extras package or combination cover on or before 30 June 2026. If you join online you must enter the promo code 12WFREEWW at the time of joining to be eligible to receive the offer. If you don’t enter the promo code you will not receive the offer. This offer is only available when you join ahm via ahm.com.au, ahm phone or ahm live chat. It is not available when you join through an aggregator. Not available in conjunction with any other ahm or third party offers. Not available for hospital only, extras only, ambulance only or overseas student health cover. Cannot be redeemed for cash. ahm may amend the offer terms and conditions and/or end this offer at any time without notice. Waiting periods may apply to hospital and/or extras cover. Annual limits on extras cover apply. If switching funds, any amount of your annual limits used while you were with your previous fund may be deducted. This offer is not available for ahm and Medibank employees. 12 weeks free Must maintain eligible hospital and extras cover continuously for 60 days from the cover start date to receive 6 weeks free. If you change to an ineligible cover during this period, 6 weeks free will not be issued. Members must maintain eligible hospital and extras cover continuously and be financial 13 months from the cover start date to be eligible to receive a further 6 weeks free. If members change to an ineligible product during this period, 6 weeks free won’t be applied. No other discount will be applied in the second year of membership.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
@@ -1252,11 +1268,23 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>up to 8 weeks free</t>
+        </is>
+      </c>
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="n"/>
-      <c r="H14" s="12" t="n"/>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>30 jun 2026</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>General - offer for new joins Available for new members on new memberships who have not held ahm hospital and/or extras cover in the last 30 days from their cover start date (unless a dependant coming off a family cover or single parent family cover). Must join and commence an ahm extras only cover on or before 30 June 2026. If you join online you must enter the promo code EXTRAS8WF at the time of joining to be eligible to receive the offer. If you don’t enter the promo code you will not receive the offer. Only available when you join via ahm.com.au, ahm phone or ahm live chat. Not available when you join through an aggregator. Not available in conjunction with any other ahm or third party offers. Not available for hospital and extras packages or combinations, hospital only, ambulance only or overseas student health cover. This offer is only available for ahm extras only health cover. Cannot be redeemed for cash. ahm may amend the offer terms and conditions and/or end this offer at any time without notice. Waiting periods may apply to hospital and/or extras cover. Annual limits on extras cover apply. If switching funds, any amount of your annual limits used while you were with your previous fund may be deducted. This offer is not available for ahm and Medibank employees. 8 weeks free Must maintain eligible extras cover continuously for 60 days from the cover start date to receive 6 weeks free. If you change to an ineligible cover during this period, 6 weeks free will not be issued. Members must maintain eligible extras cover continuously and be financial 12 months from the cover start date to be eligible to receive a further 2 weeks free. If members change to an ineligible product during this period, 2 weeks free won’t be applied. No other discount will be applied in the second year of membership. Support when you need it. message us phone us 1300 483 439</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="17" customHeight="1" thickBot="1">
       <c r="A15" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Refactored hbf, hcf, nib, bupa and finder offers
</commit_message>
<xml_diff>
--- a/comp_offer.xlsx
+++ b/comp_offer.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15760" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -641,7 +641,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col width="25.6640625" customWidth="1" min="1" max="6"/>
   </cols>
@@ -678,7 +678,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="31.95" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>medibank</t>
@@ -708,7 +708,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="16.05" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>medibank</t>
@@ -730,7 +730,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="16" customHeight="1">
+    <row r="4" ht="16.05" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>medibank</t>
@@ -754,7 +754,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1">
+    <row r="5" ht="16.05" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>medibank</t>
@@ -778,7 +778,7 @@
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
     </row>
-    <row r="6" ht="16" customHeight="1">
+    <row r="6" ht="16.05" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>medibank</t>
@@ -822,7 +822,7 @@
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" ht="16.05" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>ahm</t>
@@ -838,28 +838,28 @@
     <row r="14">
       <c r="A14" s="2" t="n"/>
     </row>
-    <row r="15" ht="16" customHeight="1">
+    <row r="15" ht="16.05" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>HCF</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
+    <row r="16" ht="16.05" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>HBF</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
+    <row r="17" ht="16.05" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>NIB</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
+    <row r="18" ht="16.05" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>BUPA</t>
@@ -878,11 +878,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.6640625" customWidth="1" style="6" min="1" max="8"/>
-    <col width="9.1640625" customWidth="1" style="6" min="9" max="9"/>
-    <col width="9.1640625" customWidth="1" style="6" min="10" max="16384"/>
+    <col width="9.109375" customWidth="1" style="6" min="9" max="16"/>
+    <col width="9.109375" customWidth="1" style="6" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -927,7 +927,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="16.05" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Medibank</t>
@@ -943,13 +943,33 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="12" t="n"/>
-      <c r="G2" s="12" t="n"/>
-      <c r="H2" s="12" t="n"/>
-    </row>
-    <row r="3" ht="16" customHeight="1">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>up to 12 weeks free</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>2&amp;6 month waiting periods on extras</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>$300 in gift cards, 30,000 live better points</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>31 july 2026 11:59pm aet</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>Hospital and Extras offer: For new members who join and start eligible combined Hospital and Extras cover from 14 May 2026 – 31 July 2026 11:59PM AET and who have not held Medibank health cover in previous 60 days (unless they are dependents coming off their parent’s cover). Must quote promo code 12WEEKSPLUS and set up direct debit when joining. Must have Australian residence . Excludes Corporate covers, Hospital only cover, Extras only cover, Overseas Visitors Health Cover, Overseas Workers Health Cover, Overseas Students Health Cover (OSHC), Ambulance Cover, ahm covers, and other selected covers. Not available to Medibank employees. Not available with any other offer. Medibank reserves the right to amend these Terms and Conditions from time to time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16.05" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Medibank</t>
@@ -987,7 +1007,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="16" customHeight="1">
+    <row r="4" ht="16.05" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Medibank</t>
@@ -1009,7 +1029,7 @@
       <c r="G4" s="12" t="n"/>
       <c r="H4" s="12" t="n"/>
     </row>
-    <row r="5" ht="16" customHeight="1">
+    <row r="5" ht="16.05" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Medibank</t>
@@ -1035,7 +1055,7 @@
       <c r="G5" s="12" t="n"/>
       <c r="H5" s="12" t="n"/>
     </row>
-    <row r="6" ht="16" customHeight="1">
+    <row r="6" ht="16.05" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Medibank</t>
@@ -1051,13 +1071,33 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="12" t="n"/>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="12" t="n"/>
-    </row>
-    <row r="7" ht="17" customHeight="1" thickBot="1">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>up to 8 weeks free</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>2&amp;6 month waiting periods on extras</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>$50 gift card, 5,000 live better rewards points</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>30 june 2026</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>Extras only offer: For new members on new memberships who join and maintain eligible extras cover by 30 June 2026 and who have not held Medibank health cover in previous 60 days (unless they are a dependent coming off their parent’s cover). Must quote promo code EXTRA8WEEKS and set up direct debit when joining. Eligible extras cover means Medibank standalone extras policies, excluding Healthy Living Extras. Offer does not apply to combined Hospital &amp; Extras covers, Corporate covers, Hospital Cover, Accident Cover, Ambulance Cover, Overseas Visitors Health Insurance, Overseas Students Health Cover (OSHC), Overseas Workers Health cover, ahm covers and other selected covers. Not available to Medibank employees. Not available with any other offer. Medibank reserves the right to amend these Terms and Conditions from time to time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16.95" customHeight="1" thickBot="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Medibank</t>
@@ -1095,7 +1135,7 @@
       </c>
       <c r="H7" s="16" t="n"/>
     </row>
-    <row r="8" ht="16" customHeight="1" thickBot="1">
+    <row r="8" ht="16.05" customHeight="1" thickBot="1">
       <c r="B8" s="7" t="n"/>
     </row>
     <row r="9">
@@ -1140,7 +1180,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
+    <row r="10" ht="16.05" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>AHM</t>
@@ -1178,7 +1218,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" ht="16.05" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>AHM</t>
@@ -1208,7 +1248,7 @@
       </c>
       <c r="H11" s="12" t="n"/>
     </row>
-    <row r="12" ht="16" customHeight="1">
+    <row r="12" ht="16.05" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>AHM</t>
@@ -1230,7 +1270,7 @@
       <c r="G12" s="12" t="n"/>
       <c r="H12" s="12" t="n"/>
     </row>
-    <row r="13" ht="16" customHeight="1">
+    <row r="13" ht="16.05" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>AHM</t>
@@ -1252,7 +1292,7 @@
       <c r="G13" s="12" t="n"/>
       <c r="H13" s="12" t="n"/>
     </row>
-    <row r="14" ht="16" customHeight="1">
+    <row r="14" ht="16.05" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
           <t>AHM</t>
@@ -1282,11 +1322,11 @@
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>General - offer for new joins Available for new members on new memberships who have not held ahm hospital and/or extras cover in the last 30 days from their cover start date (unless a dependant coming off a family cover or single parent family cover). Must join and commence an ahm extras only cover on or before 30 June 2026. If you join online you must enter the promo code EXTRAS8WF at the time of joining to be eligible to receive the offer. If you don’t enter the promo code you will not receive the offer. Only available when you join via ahm.com.au, ahm phone or ahm live chat. Not available when you join through an aggregator. Not available in conjunction with any other ahm or third party offers. Not available for hospital and extras packages or combinations, hospital only, ambulance only or overseas student health cover. This offer is only available for ahm extras only health cover. Cannot be redeemed for cash. ahm may amend the offer terms and conditions and/or end this offer at any time without notice. Waiting periods may apply to hospital and/or extras cover. Annual limits on extras cover apply. If switching funds, any amount of your annual limits used while you were with your previous fund may be deducted. This offer is not available for ahm and Medibank employees. 8 weeks free Must maintain eligible extras cover continuously for 60 days from the cover start date to receive 6 weeks free. If you change to an ineligible cover during this period, 6 weeks free will not be issued. Members must maintain eligible extras cover continuously and be financial 12 months from the cover start date to be eligible to receive a further 2 weeks free. If members change to an ineligible product during this period, 2 weeks free won’t be applied. No other discount will be applied in the second year of membership. Support when you need it. message us phone us 1300 483 439</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1" thickBot="1">
+          <t>General - offer for new joins Available for new members on new memberships who have not held ahm hospital and/or extras cover in the last 30 days from their cover start date (unless a dependant coming off a family cover or single parent family cover). Must join and commence an ahm extras only cover on or before 30 June 2026. If you join online you must enter the promo code EXTRAS8WF at the time of joining to be eligible to receive the offer. If you don’t enter the promo code you will not receive the offer. Only available when you join via ahm.com.au, ahm phone or ahm live chat. Not available when you join through an aggregator. Not available in conjunction with any other ahm or third party offers. Not available for hospital and extras packages or combinations, hospital only, ambulance only or overseas student health cover. This offer is only available for ahm extras only health cover. Cannot be redeemed for cash. ahm may amend the offer terms and conditions and/or end this offer at any time without notice. Waiting periods may apply to hospital and/or extras cover. Annual limits on extras cover apply. If switching funds, any amount of your annual limits used while you were with your previous fund may be deducted. This offer is not available for ahm and Medibank employees. 8 weeks free Must maintain eligible extras cover continuously for 60 days from the cover start date to receive 6 weeks free. If you change to an ineligible cover during this period, 6 weeks free will not be issued. Members must maintain eligible extras cover continuously and be financial 12 months from the cover start date to be eligible to receive a further 2 weeks free. If members change to an ineligible product during this period, 2 weeks free won’t be applied. No other discount will be applied in the second year of membership. Support when you need it. message us phone us 1300 537 636</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16.95" customHeight="1" thickBot="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
           <t>AHM</t>
@@ -1316,7 +1356,7 @@
       </c>
       <c r="H15" s="16" t="n"/>
     </row>
-    <row r="16" ht="16" customHeight="1" thickBot="1">
+    <row r="16" ht="16.05" customHeight="1" thickBot="1">
       <c r="B16" s="7" t="n"/>
     </row>
     <row r="17">
@@ -1361,7 +1401,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
+    <row r="18" ht="16.05" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
           <t>BUPA</t>
@@ -1389,21 +1429,21 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Code: 10WEEKSFREE | Everyday Rewards: Code: EVERYDAY120</t>
+          <t>Code: 10WEEKSFREE</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>10 June 2026 | Everyday Rewards: 8 July 2026</t>
+          <t>10 June 2026</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>Eligibility: New Members Only | Waiting Periods: Waive The 2 &amp; 6 Month Waiting Periods On Extras* | Fulfilment: 10 Weeks Free Applied Over 2 Years | Annual Payers: 3 Years For Annual Payers | Offer Period: Join By 10 June 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
+          <t>Eligibility: New Members Only | Waiting Periods: Waive The 2 &amp; 6 Month Waiting Periods On Extras!* Use Promo Code 10Weeksfree We’Ll Even Waive The 2 &amp; 6 Month Waiting Periods On Extras!* New Members Only | Fulfilment: 10 Weeks Free Applied Over 2 Years | Annual Payers: 3 Years For Annual Payers | Offer Period: Join By 10 June 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16.05" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>BUPA</t>
@@ -1437,7 +1477,7 @@
       </c>
       <c r="H19" s="12" t="n"/>
     </row>
-    <row r="20" ht="16" customHeight="1">
+    <row r="20" ht="16.05" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
           <t>BUPA</t>
@@ -1475,7 +1515,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
+    <row r="21" ht="16.05" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>BUPA</t>
@@ -1497,7 +1537,7 @@
       <c r="G21" s="12" t="n"/>
       <c r="H21" s="12" t="n"/>
     </row>
-    <row r="22" ht="16" customHeight="1">
+    <row r="22" ht="16.05" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
           <t>BUPA</t>
@@ -1515,15 +1555,23 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>No current offer</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="12" t="n"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>2 &amp; 6 month waits waived</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Code: 6WEEKSCORP</t>
+        </is>
+      </c>
       <c r="G22" s="12" t="n"/>
       <c r="H22" s="12" t="n"/>
     </row>
-    <row r="23" ht="17" customHeight="1" thickBot="1">
+    <row r="23" ht="16.95" customHeight="1" thickBot="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
           <t>BUPA</t>
@@ -1545,7 +1593,7 @@
       <c r="G23" s="16" t="n"/>
       <c r="H23" s="16" t="n"/>
     </row>
-    <row r="24" ht="16" customHeight="1" thickBot="1">
+    <row r="24" ht="16.05" customHeight="1" thickBot="1">
       <c r="B24" s="7" t="n"/>
     </row>
     <row r="25">
@@ -1590,7 +1638,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1">
+    <row r="26" ht="16.05" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
           <t>NIB</t>
@@ -1628,7 +1676,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1">
+    <row r="27" ht="16.05" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>NIB</t>
@@ -1650,7 +1698,7 @@
       <c r="G27" s="12" t="n"/>
       <c r="H27" s="12" t="n"/>
     </row>
-    <row r="28" ht="16" customHeight="1">
+    <row r="28" ht="16.05" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
           <t>NIB</t>
@@ -1684,7 +1732,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1">
+    <row r="29" ht="16.05" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>NIB</t>
@@ -1706,7 +1754,7 @@
       <c r="G29" s="12" t="n"/>
       <c r="H29" s="12" t="n"/>
     </row>
-    <row r="30" ht="16" customHeight="1">
+    <row r="30" ht="16.05" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
           <t>NIB</t>
@@ -1724,15 +1772,23 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>No current offer</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n"/>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>2 &amp; 6 month waits waived</t>
+        </is>
+      </c>
       <c r="F30" s="12" t="n"/>
       <c r="G30" s="12" t="n"/>
-      <c r="H30" s="12" t="n"/>
-    </row>
-    <row r="31" ht="17" customHeight="1" thickBot="1">
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>Eligibility: Available To New Members With Australian Residency | Offer Period: Join By 30 June 2026 | Waiting Periods: Skip The 2 &amp; 6 Month Wait On Extras | Fulfilment: 3Rd And 13Th Month Of Membership</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16.95" customHeight="1" thickBot="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
           <t>NIB</t>
@@ -1754,7 +1810,7 @@
       <c r="G31" s="16" t="n"/>
       <c r="H31" s="16" t="n"/>
     </row>
-    <row r="32" ht="16" customHeight="1" thickBot="1">
+    <row r="32" ht="16.05" customHeight="1" thickBot="1">
       <c r="B32" s="7" t="n"/>
     </row>
     <row r="33">
@@ -1799,7 +1855,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
+    <row r="34" ht="16.05" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
           <t>HCF</t>
@@ -1815,13 +1871,17 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D34" s="4" t="n"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>No current offer</t>
+        </is>
+      </c>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="12" t="n"/>
       <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
     </row>
-    <row r="35" ht="16" customHeight="1">
+    <row r="35" ht="16.05" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>HCF</t>
@@ -1845,9 +1905,13 @@
         </is>
       </c>
       <c r="G35" s="12" t="n"/>
-      <c r="H35" s="12" t="n"/>
-    </row>
-    <row r="36" ht="16" customHeight="1">
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>basic/bronze/silver: HCF Loyalty Program T&amp;C: ELIGIBLE MEMBERS AND MEMBERSHIP TIERS 5. An Eligible Member is an HCF Member: (a) who has held an Eligible Product for at least one week; and (a) who holds an Eligible Product and: (i) the policy for that Eligible Product is active and financial and not in arrears; and (i) meets the criteria for recognition (set out in clauses 6 – 10 below) under HCF Thank You as an Opal, Emerald, Ruby or Diamond Membership Tier. 6. HCF members will not be eligible to access HCF Thank You if they only hold Overseas Visitors Health Cover. However, if such HCF members subsequently take up an Eligible Product, they will have their HCF membership tenure on their Overseas Visitors Health Cover product recognised for the purposes of calculating their HCF Thank You Membership Tier and gain access to HCF Thank You. 7. If an Eligible Member on a specific policy leaves the policy and establishes their own policy within 90 days, they will retain the Membership Tier of their previous policy. For example, if a teenager is covered under their parent’s policy with Diamond tier status, and they leave that policy to immediately establish their own policy with an Eligible Product, they will retain Diamond tier status on their new policy. 8. If the primary policy holder dies, any other Eligible Members on that policy will inherit the same Membership Tier as the primary policy holder, even if they move to another existing or new policy, as long as they remain on an Eligible Product. 9. If existing Eligible Members combine their policies into one, the highest Membership Tier from the Eligible Members will be assigned to each them, even if the primary policy holder is only otherwise eligible for a lower tier. 10. An Eligible Member who: (a) changes their product and no longer holds an Eligible Product will no longer be eligible for access to HCF Thank You. If they re-instate their policy to an Eligible Product any time during the course of their policy, their tenure on the ineligible product will count towards calculation of their HCF Thank You Membership Tier. (b) has their policy terminated, or ceases to be an HCF Member will no longer be eligible for access to HCF Thank You. If they reinstate their policy to an Eligible Product within 90 days of their policy being terminated or ceasing to be a member, their previous tenure will continue to accrue and they will retain their previous Membership Tier. If they re-join HCF on an Eligible Product after 90 days, their previous tenure will not be counted for assigning a Membership Tier. (c) is granted an overseas suspension, will not continue to accrue tenure towards their HCF Thank You Membership Tier while the overseas suspension is in place. (d) is granted unemployment and sickness, hardship or natural disaster suspension will continue to accrue tenure towards their HCF Thank You Membership Tier while the suspension is in place. 11. HCF reserves the right to allocate, at its discretion, a higher Membership Tier to an Eligible Member than would ordinarily be available to that Eligible Member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16.05" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
           <t>HCF</t>
@@ -1863,13 +1927,17 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D36" s="4" t="n"/>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>No current offer</t>
+        </is>
+      </c>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="12" t="n"/>
       <c r="G36" s="12" t="n"/>
       <c r="H36" s="12" t="n"/>
     </row>
-    <row r="37" ht="16" customHeight="1">
+    <row r="37" ht="16.05" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>HCF</t>
@@ -1893,9 +1961,13 @@
         </is>
       </c>
       <c r="G37" s="12" t="n"/>
-      <c r="H37" s="12" t="n"/>
-    </row>
-    <row r="38" ht="16" customHeight="1">
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>basic/bronze/silver: HCF Loyalty Program T&amp;C: ELIGIBLE MEMBERS AND MEMBERSHIP TIERS 5. An Eligible Member is an HCF Member: (a) who has held an Eligible Product for at least one week; and (a) who holds an Eligible Product and: (i) the policy for that Eligible Product is active and financial and not in arrears; and (i) meets the criteria for recognition (set out in clauses 6 – 10 below) under HCF Thank You as an Opal, Emerald, Ruby or Diamond Membership Tier. 6. HCF members will not be eligible to access HCF Thank You if they only hold Overseas Visitors Health Cover. However, if such HCF members subsequently take up an Eligible Product, they will have their HCF membership tenure on their Overseas Visitors Health Cover product recognised for the purposes of calculating their HCF Thank You Membership Tier and gain access to HCF Thank You. 7. If an Eligible Member on a specific policy leaves the policy and establishes their own policy within 90 days, they will retain the Membership Tier of their previous policy. For example, if a teenager is covered under their parent’s policy with Diamond tier status, and they leave that policy to immediately establish their own policy with an Eligible Product, they will retain Diamond tier status on their new policy. 8. If the primary policy holder dies, any other Eligible Members on that policy will inherit the same Membership Tier as the primary policy holder, even if they move to another existing or new policy, as long as they remain on an Eligible Product. 9. If existing Eligible Members combine their policies into one, the highest Membership Tier from the Eligible Members will be assigned to each them, even if the primary policy holder is only otherwise eligible for a lower tier. 10. An Eligible Member who: (a) changes their product and no longer holds an Eligible Product will no longer be eligible for access to HCF Thank You. If they re-instate their policy to an Eligible Product any time during the course of their policy, their tenure on the ineligible product will count towards calculation of their HCF Thank You Membership Tier. (b) has their policy terminated, or ceases to be an HCF Member will no longer be eligible for access to HCF Thank You. If they reinstate their policy to an Eligible Product within 90 days of their policy being terminated or ceasing to be a member, their previous tenure will continue to accrue and they will retain their previous Membership Tier. If they re-join HCF on an Eligible Product after 90 days, their previous tenure will not be counted for assigning a Membership Tier. (c) is granted an overseas suspension, will not continue to accrue tenure towards their HCF Thank You Membership Tier while the overseas suspension is in place. (d) is granted unemployment and sickness, hardship or natural disaster suspension will continue to accrue tenure towards their HCF Thank You Membership Tier while the suspension is in place. 11. HCF reserves the right to allocate, at its discretion, a higher Membership Tier to an Eligible Member than would ordinarily be available to that Eligible Member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16.05" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
           <t>HCF</t>
@@ -1911,13 +1983,17 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D38" s="4" t="n"/>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>No current offer</t>
+        </is>
+      </c>
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="12" t="n"/>
       <c r="G38" s="12" t="n"/>
       <c r="H38" s="12" t="n"/>
     </row>
-    <row r="39" ht="17" customHeight="1" thickBot="1">
+    <row r="39" ht="16.95" customHeight="1" thickBot="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
           <t>HCF</t>
@@ -1941,9 +2017,13 @@
         </is>
       </c>
       <c r="G39" s="16" t="n"/>
-      <c r="H39" s="16" t="n"/>
-    </row>
-    <row r="40" ht="16" customHeight="1" thickBot="1">
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>HCF Loyalty Program T&amp;C: ELIGIBLE MEMBERS AND MEMBERSHIP TIERS 5. An Eligible Member is an HCF Member: (a) who has held an Eligible Product for at least one week; and (a) who holds an Eligible Product and: (i) the policy for that Eligible Product is active and financial and not in arrears; and (i) meets the criteria for recognition (set out in clauses 6 – 10 below) under HCF Thank You as an Opal, Emerald, Ruby or Diamond Membership Tier. 6. HCF members will not be eligible to access HCF Thank You if they only hold Overseas Visitors Health Cover. However, if such HCF members subsequently take up an Eligible Product, they will have their HCF membership tenure on their Overseas Visitors Health Cover product recognised for the purposes of calculating their HCF Thank You Membership Tier and gain access to HCF Thank You. 7. If an Eligible Member on a specific policy leaves the policy and establishes their own policy within 90 days, they will retain the Membership Tier of their previous policy. For example, if a teenager is covered under their parent’s policy with Diamond tier status, and they leave that policy to immediately establish their own policy with an Eligible Product, they will retain Diamond tier status on their new policy. 8. If the primary policy holder dies, any other Eligible Members on that policy will inherit the same Membership Tier as the primary policy holder, even if they move to another existing or new policy, as long as they remain on an Eligible Product. 9. If existing Eligible Members combine their policies into one, the highest Membership Tier from the Eligible Members will be assigned to each them, even if the primary policy holder is only otherwise eligible for a lower tier. 10. An Eligible Member who: (a) changes their product and no longer holds an Eligible Product will no longer be eligible for access to HCF Thank You. If they re-instate their policy to an Eligible Product any time during the course of their policy, their tenure on the ineligible product will count towards calculation of their HCF Thank You Membership Tier. (b) has their policy terminated, or ceases to be an HCF Member will no longer be eligible for access to HCF Thank You. If they reinstate their policy to an Eligible Product within 90 days of their policy being terminated or ceasing to be a member, their previous tenure will continue to accrue and they will retain their previous Membership Tier. If they re-join HCF on an Eligible Product after 90 days, their previous tenure will not be counted for assigning a Membership Tier. (c) is granted an overseas suspension, will not continue to accrue tenure towards their HCF Thank You Membership Tier while the overseas suspension is in place. (d) is granted unemployment and sickness, hardship or natural disaster suspension will continue to accrue tenure towards their HCF Thank You Membership Tier while the suspension is in place. 11. HCF reserves the right to allocate, at its discretion, a higher Membership Tier to an Eligible Member than would ordinarily be available to that Eligible Member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16.05" customHeight="1" thickBot="1">
       <c r="A40" s="17" t="n"/>
       <c r="B40" s="7" t="n"/>
       <c r="F40" s="18" t="n"/>
@@ -1990,7 +2070,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16" customHeight="1">
+    <row r="42" ht="16.05" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
           <t>HBF</t>
@@ -2006,13 +2086,29 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>up to 14 weeks free</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>serve no waits on eligible extras</t>
+        </is>
+      </c>
       <c r="F42" s="12" t="n"/>
-      <c r="G42" s="12" t="n"/>
-      <c r="H42" s="12" t="n"/>
-    </row>
-    <row r="43" ht="16" customHeight="1">
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>30 july 2026</t>
+        </is>
+      </c>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>Promotional offer: Up to 14 Weeks Free &amp; No Waits on Eligible Extras new member offer with Competition (13 May 2026 – 30 July 2026) Terms and conditions Eligible covers: The offer is available on the following eligible HBF hospital and extras covers when purchased together in one transaction: Hospital: Basic Hospital Accident Only Basic Hospital Plus Basic Hospital Plus Elevate Lite Bronze Hospital Plus Bronze Hospital Plus Essential Silver Hospital Silver Hospital Silver Hospital Plus Gold Hospital Elevate Extras: Smart Start Extras Basic Extras Value 50 Flex 50 Flex 60 Core Extras Complete 60 Top 70 To be eligible to receive up to 14 weeks free cover and no waits on eligible extras: You must start your cover between 12.01am AWST, Wednesday 13 May 2026 and 11.59pm AWST, Thursday 30 July 2026 on eligible HBF Hospital and Extras cover purchased together in a single transaction. Maintain continuous eligible HBF Hospital and Extras cover until the offer is fulfilled in its entirety after 26 months. To receive 6 weeks free cover, you must hold your eligible HBF Hospital and Extras cover for at least 31 days from the start date of your policy. To receive a further 4 weeks free cover, you must hold your eligible HBF Hospital and Extras cover for 13 months from the start date of your policy. To receive the final 4 weeks free cover, you must hold your eligible HBF Hospital and Extras cover for 26 months from the start date of your policy. Be a new HBF member or have not held an HBF branded policy (hospital and/or extras, including urgent and essential ambulance) in the last 60 days (dependants coming off a family policy and partners coming off a couples/ family policy are eligible). Pay premiums monthly or fortnightly via direct debit and ensure payments are up to date at the time of fulfilment. Provide a valid email address. If joining online at hbf.com.au, select ‘Up to 14 weeks free plus no waits on eligible extras promotion’. If joining via phone or in branch, request to receive ‘Up to 14 weeks free plus no waits on eligible extras promotion’. The offer does not apply to: Members who start their cover before 12.01am AWST, Wednesday 13 May 2026 and after 11.59pm AWST, Thursday 30 July 2026. Current HBF members (dependants coming off a family policy and partners coming off a couples/family policy are eligible). Members who pay premiums quarterly, half-yearly, or annually. Members who are not paying by direct debit. HBF, see-u and QCHF employees and their immediate family members eligible for HBF staff discounts. Current HBF members (dependants coming off a family policy and partners coming off a couples/family policy are eligible) or those who have redeemed another HBF promotional or save offer, or corporate discount, in the last 12 months, excluding direct debit discount. Members who join on a corporate policy eligible for a corporate discount are ineligible for this offer. Members who terminate or suspend their cover during the promotional period. Members who join via a third-party broker or aggregator (excluding Finder). Fulfilment of the 14 weeks free cover will be applied over 26 months: 6 weeks free cover will be applied to your policy at the next billing cycle after you have held eligible cover for 31 consecutive days from the start date of your policy. A further 4 weeks free cover will be applied to your policy at the next billing cycle after you have held eligible cover for 13 months from the start date of your policy. The final 4 weeks free cover will be applied to your policy at the next billing cycle after you have held eligible cover for 26 months from the start date of your policy. A member may change their level of eligible cover during the offer. The value of the weeks free cover will apply to the level of eligible cover held at each fulfilment period. Direct debits during the free periods will be adjusted, and your account will show your policy as paid until the end of each free cover period. Your direct debit schedule will not be altered due to applying the free cover. If you fail any eligibility checks, all future fulfilments will be removed. Weeks Free cannot be exchanged for cash in the form of a refund due to policy cancellation. Fulfilment of the 2-month waived waits on Extras HBF will waive the 2-month waiting period on eligible HBF Extras of the product you selected upon joining, effective from the policy start date. However, claims will only be paid once your policy is financial (i.e., payment has been made). You may submit a manual claim before your policy becomes financial and it will be honoured once your policy is up to date. Waiting periods for extras that are longer than 2 months and all hospital treatment waiting periods, still apply. If you’re switching from another fund, your available limits will be adjusted to take into account any extras benefits you have received this calendar year from your previous fund. This may affect your ability to claim. Reservation of Rights: HBF reserves the right to amend, add to, or end this offer, along with its terms and conditions, at any time without notice. Changes made will be effective immediately and will be reflected in the Terms and Conditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16.05" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>HBF</t>
@@ -2040,21 +2136,21 @@
       </c>
       <c r="F43" s="12" t="inlineStr">
         <is>
-          <t>bronze/silver/gold: $500 Reward (Finder Rewards) T&amp;Cs apply</t>
+          <t>$500 Reward (Finder Rewards) T&amp;Cs apply</t>
         </is>
       </c>
       <c r="G43" s="12" t="inlineStr">
         <is>
-          <t>basic: 30 jul 2026 | bronze/silver/gold: 30 jul 2026 | Finder Rewards: 30 Jun 2026</t>
+          <t>30 jul 2026 | Finder Rewards: 30 Jun 2026</t>
         </is>
       </c>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>bronze/silver/gold: Finder Reward: Eligibility: Available to new HBF customers or customers who have not held HBF hospital and/or extras cover (including urgent ambulance) within the last 60 days (excluding eligible dependents coming off a family policy) | Excluded Covers: Basic Hospital Accident Only, Essential Ambulance, Urgent Ambulance and Ambulance Care | Payment Requirement: Premiums must be paid monthly or fortnightly via direct debit | Reward Fulfilment Date: On or before 29 January 2027 | Stackable Offer: This Finder Rewards promotion may be combined with eligible HBF new member promotions, including up to 14 weeks free on selected combined Hospital &amp; Extras policies, provided all eligibility criteria for both offers are met.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16" customHeight="1">
+          <t>Finder Reward: Eligibility: Available to new HBF customers or customers who have not held HBF hospital and/or extras cover (including urgent ambulance) within the last 60 days (excluding eligible dependents coming off a family policy) | Excluded Covers: Basic Hospital Accident Only, Essential Ambulance, Urgent Ambulance and Ambulance Care | Payment Requirement: Premiums must be paid monthly or fortnightly via direct debit | Reward Fulfilment Date: On or before 29 January 2027 | Stackable Offer: This Finder Rewards promotion may be combined with eligible HBF new member promotions, including up to 14 weeks free on selected combined Hospital &amp; Extras policies, provided all eligibility criteria for both offers are met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16.05" customHeight="1">
       <c r="A44" s="11" t="inlineStr">
         <is>
           <t>HBF</t>
@@ -2070,13 +2166,25 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D44" s="4" t="n"/>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>up to 6 weeks free</t>
+        </is>
+      </c>
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="12" t="n"/>
-      <c r="G44" s="12" t="n"/>
-      <c r="H44" s="12" t="n"/>
-    </row>
-    <row r="45" ht="16" customHeight="1">
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>30 june 2026</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>Promotional offer: 6 Weeks Free (Hospital Only) (1 April 2026 – 30 June 2026) Terms and conditions Eligible covers: The offer is available on the following eligible HBF hospital cover: Basic Hospital Accident Only Basic Hospital Plus Basic Hospital Plus Elevate Lite Bronze Hospital Plus Bronze Hospital Plus Silver Hospital Silver Hospital Plus Essential Silver Hospital Gold Hospital Elevate To be eligible to receive 6 weeks free: You must start your cover between 12.01am AWST, Wednesday 1 April 2026 and 11.59pm AWST, Tuesday 30 June 2026 on eligible hospital only cover purchased in a single transaction. Maintain continuous eligible HBF hospital cover until the offer is fulfilled in its entirety at 31 days of continuous cover. To receive 6 weeks free cover, you must hold your eligible HBF hospital cover for 31 days from the start date of your policy. Be a new HBF member or have not held an HBF branded policy (hospital and/or extras, including urgent ambulance) in the last 60 days (dependents coming of a family policy and partners coming off a couples/ family policy are eligible). Pay premiums monthly or fortnightly via direct debit and ensure payments are up to date at the time of fulfilment. Provide a valid email address. If joining online at hbf.com.au - select ‘6 weeks free promotion’. If joining via phone or in branch - request to receive ‘6 weeks free promotion’. The offer does not apply to: Members who start their cover before 12.01am AWST, Wednesday 1 April 2026 and after 11.59pm AWST, Tuesday 30 June 2026. Members taking out extras only cover or combined cover. Current HBF members, holding an HBF Health branded product (dependents coming off a family policy and partners coming off a couples/family policy are eligible) or those who have redeemed another HBF promotional or save offer, or corporate discount, in the last 12 months, excluding direct debit discount. Members who pay premiums quarterly, half-yearly, or annually. Members who are not paying by direct debit. HBF, see-u and QCHF employees and their immediate family members eligible for HBF staff discounts. Members who terminate or suspend their cover during the promotional period. Members who join via a third-party broker or aggregator (excluding Finder). Fulfilment of the 6 weeks free cover: 6 weeks free cover will be applied to your policy at the next billing cycle after you have held eligible cover for 31 consecutive days from the start date of your policy. A member may change their level of eligible hospital cover during the offer, the weeks free cover will apply to the level of hospital cover held at the specific fulfilment period. Direct debits during this free period will be amended and your account will show your policy as paid until the end of the free week periods. Your direct debit schedule will not be altered due to applying the free cover. If you fail any eligibility checks, all future fulfilments will be removed. The 6 weeks free offer is not redeemable for cash. Reservation of Rights: HBF reserves the right to amend, add to, or end this offer, along with its terms and conditions, at any time without notice. Changes made will be effective immediately and will be reflected in the Terms and Conditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="16.05" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>HBF</t>
@@ -2114,7 +2222,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1">
+    <row r="46" ht="16.05" customHeight="1">
       <c r="A46" s="11" t="inlineStr">
         <is>
           <t>HBF</t>
@@ -2130,12 +2238,29 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>up to 6 weeks free</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>no waits on eligible extras</t>
+        </is>
+      </c>
       <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-    </row>
-    <row r="47" ht="17" customHeight="1" thickBot="1">
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>30 june 2026</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Promotional offer: 6 weeks free (extras only) + Waived Waits (1 April 2026 – 30 June 2026) Terms and conditions Eligible covers: The offer is available on the following eligible HBF extras cover: Smart Start Extras Basic Extras Value 50 Flex 50 Flex 60 Core Extras Complete 60 Top 70 To be eligible to receive 6 weeks free and waived waits: You must start your cover between 12.01am AWST, Wednesday 1 April 2026 and 11.59pm AWST, Tuesday 30 June 2026 on eligible extras only cover purchased in a single transaction. Maintain continuous eligible HBF extras cover until the offer is fulfilled in its entirety at 31 days of continuous cover. To receive 6 weeks free cover, you must hold your eligible HBF Extras cover for 31 days from the start date of your policy. Be a new HBF member or have not held an HBF branded policy (hospital and/or extras, including urgent ambulance) in the last 60 days (dependents coming of a family policy and partners coming off a couples/ family policy are eligible). Pay premiums monthly or fortnightly via direct debit and ensure payments are up to date at the time of fulfilment. Provide a valid email address. If joining online at hbf.com.au - select ‘6 weeks free promotion’. If joining via phone or in branch - request to receive ‘6 weeks free promotion’. The offer does not apply to: Members who start their cover before 12.01am AWST, Wednesday 1 April 2026 and 11.59pm AWST, Tuesday 30 June 2026. Members taking out hospital cover or combined cover. Current HBF members, holding an HBF Health branded product (dependents coming off a family policy and partners coming off a couples/family policy are eligible) or those who have redeemed another HBF promotional or save offer, or corporate discount, in the last 12 months, excluding direct debit discount. Members who pay premiums quarterly, half-yearly, or annually. Members who are not paying by direct debit. HBF, see-u and QCHF employees and their immediate family members eligible for HBF staff discounts. Members who terminate or suspend their cover during the promotional period. Members who join via a third-party broker or aggregator (excluding Finder). Fulfilment of the 6 weeks free cover: 6 weeks free cover will be applied to your policy at the next billing cycle after you have held eligible cover for 31 consecutive days from the start date of your policy. A member may change their level of eligible extras cover during the offer, the weeks free cover will apply to the level of extras cover held at the specific fulfilment period. Direct debits during this free period will be amended and your account will show your policy as paid until the end of the free week periods. Your direct debit schedule will not be altered due to applying the free cover. If you fail any eligibility checks, all future fulfilments will be removed. The 6 weeks free offer is not redeemable for cash. Fulfilment of 2-month waived waits on Extras: HBF will waive the 2-month waiting period on eligible Extras of the product you selected upon joining, effective from the policy start date. However, claims will only be paid once your policy is financial (i.e., payment has been made). You may submit a manual claim before your policy becomes financial and it will be honoured once your policy is up to date. Waiting periods for extras that are longer than 2 months still apply. If you are switching from another fund, your available limits will be adjusted to take into account any extras benefits you have received this calendar year from your previous fund. This may affect your ability to claim. Reservation of Rights: HBF reserves the right to amend, add to, or end this offer, along with its terms and conditions, at any time without notice. Changes made will be effective immediately and will be reflected in the Terms and Conditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="16.95" customHeight="1" thickBot="1">
       <c r="A47" s="14" t="inlineStr">
         <is>
           <t>HBF</t>

</xml_diff>